<commit_message>
#18 eSpark and JLCPCB BOM Addition Completed
</commit_message>
<xml_diff>
--- a/BOM/JLCPCB-BOM.xlsx
+++ b/BOM/JLCPCB-BOM.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\matthewgraff-arduinomegapcb\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F64132A-8E33-481C-9017-57840EB94A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="268">
   <si>
     <t>Comment</t>
   </si>
@@ -58,6 +57,9 @@
     <t>47uF</t>
   </si>
   <si>
+    <t>2.2uF</t>
+  </si>
+  <si>
     <t>PESD5V0H1BSFYL</t>
   </si>
   <si>
@@ -133,6 +135,15 @@
     <t>Yellow</t>
   </si>
   <si>
+    <t>DNP</t>
+  </si>
+  <si>
+    <t>OLED Module</t>
+  </si>
+  <si>
+    <t>TEST POINT</t>
+  </si>
+  <si>
     <t>MMBT3904M</t>
   </si>
   <si>
@@ -187,6 +198,15 @@
     <t>100K</t>
   </si>
   <si>
+    <t>250R</t>
+  </si>
+  <si>
+    <t>680R</t>
+  </si>
+  <si>
+    <t>Solder Bridge</t>
+  </si>
+  <si>
     <t>Tactile Switch</t>
   </si>
   <si>
@@ -220,6 +240,9 @@
     <t>CP2102N-A02-GQFN24R</t>
   </si>
   <si>
+    <t>LMV321AIDBVR</t>
+  </si>
+  <si>
     <t>X322516MLB4SI</t>
   </si>
   <si>
@@ -229,7 +252,7 @@
     <t>C1</t>
   </si>
   <si>
-    <t>C2, C7, C9, C10, C12, C13, C19, C20, C21, C22, C29, C30, C31, C32, C33, C34, C35, C37, C40, C41, C44, C45, C46, C47, C48, C49, C51, C54</t>
+    <t>C2, C7, C9, C10, C12, C13, C19, C20, C21, C22, C29, C30, C31, C32, C33, C34, C35, C37, C40, C41, C44, C45, C46, C47, C48, C49, C51, C54, C56, C57</t>
   </si>
   <si>
     <t>C3, C5</t>
@@ -244,7 +267,7 @@
     <t>C11, C14, C15, C16, C17, C18, C23, C24, C25, C26, C27, C28</t>
   </si>
   <si>
-    <t>C38</t>
+    <t>C38, C55</t>
   </si>
   <si>
     <t>C39</t>
@@ -259,6 +282,9 @@
     <t>C53</t>
   </si>
   <si>
+    <t>C58, C59</t>
+  </si>
+  <si>
     <t>D1, D2, D3, D17, D18, D23, D24</t>
   </si>
   <si>
@@ -337,6 +363,15 @@
     <t>LED4, LED6, LED8, LED9</t>
   </si>
   <si>
+    <t>LED7</t>
+  </si>
+  <si>
+    <t>LED10</t>
+  </si>
+  <si>
+    <t>P1, P2, P3, P4, P5, P6</t>
+  </si>
+  <si>
     <t>Q1, Q2, Q3, Q4</t>
   </si>
   <si>
@@ -346,7 +381,7 @@
     <t>R2</t>
   </si>
   <si>
-    <t>R3, R8, R9, R12, R13, R14, R15, R18, R19, R24, R38, R39, R40</t>
+    <t>R3, R8, R9, R12, R13, R14, R15, R18, R19, R24, R38, R39, R40, R49</t>
   </si>
   <si>
     <t>R4</t>
@@ -394,6 +429,12 @@
     <t>R48</t>
   </si>
   <si>
+    <t>R50</t>
+  </si>
+  <si>
+    <t>R51, R52</t>
+  </si>
+  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -427,6 +468,9 @@
     <t>U13</t>
   </si>
   <si>
+    <t>U14, U15</t>
+  </si>
+  <si>
     <t>X1</t>
   </si>
   <si>
@@ -508,6 +552,12 @@
     <t>LED-0603</t>
   </si>
   <si>
+    <t>ZIO-101954</t>
+  </si>
+  <si>
+    <t>Test-point</t>
+  </si>
+  <si>
     <t>SOT-723</t>
   </si>
   <si>
@@ -517,6 +567,9 @@
     <t>Res-0402</t>
   </si>
   <si>
+    <t>Res-1206</t>
+  </si>
+  <si>
     <t>TL3301NF160QG</t>
   </si>
   <si>
@@ -544,6 +597,9 @@
     <t>24-QFN (4x4)</t>
   </si>
   <si>
+    <t>SOT-23-5</t>
+  </si>
+  <si>
     <t>SMD3225-4P</t>
   </si>
   <si>
@@ -571,9 +627,6 @@
     <t>C14664</t>
   </si>
   <si>
-    <t>C441758</t>
-  </si>
-  <si>
     <t>C105621</t>
   </si>
   <si>
@@ -583,6 +636,9 @@
     <t>C136280</t>
   </si>
   <si>
+    <t>C326581</t>
+  </si>
+  <si>
     <t>C477989</t>
   </si>
   <si>
@@ -637,9 +693,6 @@
     <t>C492442</t>
   </si>
   <si>
-    <t>C492441</t>
-  </si>
-  <si>
     <t>C597972</t>
   </si>
   <si>
@@ -709,6 +762,12 @@
     <t>C137715</t>
   </si>
   <si>
+    <t>C3033906</t>
+  </si>
+  <si>
+    <t>C112310</t>
+  </si>
+  <si>
     <t>C273526</t>
   </si>
   <si>
@@ -742,23 +801,35 @@
     <t>C969151</t>
   </si>
   <si>
+    <t>C484730</t>
+  </si>
+  <si>
     <t>C13738</t>
   </si>
   <si>
+    <t>SB1, SB2, SB8</t>
+  </si>
+  <si>
+    <t>C526997</t>
+  </si>
+  <si>
+    <t>C69679</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>C114765</t>
   </si>
   <si>
     <t>C60491</t>
-  </si>
-  <si>
-    <t>C69679</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -787,6 +858,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -808,7 +887,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -890,37 +969,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -946,10 +999,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1237,9 +1287,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1253,13 +1303,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1267,13 +1317,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="36" x14ac:dyDescent="0.25">
@@ -1281,13 +1331,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1295,13 +1345,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>178</v>
+        <v>153</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1309,13 +1359,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1323,13 +1373,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>180</v>
+        <v>155</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1337,13 +1387,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1351,13 +1401,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>182</v>
+        <v>152</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1365,13 +1415,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>183</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1379,13 +1429,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>184</v>
+        <v>152</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1393,13 +1443,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1407,13 +1457,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1421,13 +1471,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1435,13 +1485,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>188</v>
+        <v>158</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1449,13 +1499,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1463,13 +1513,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>190</v>
+        <v>160</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1477,13 +1527,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>191</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1491,13 +1541,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>192</v>
+        <v>161</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1505,13 +1555,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1519,13 +1569,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>194</v>
+        <v>163</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1533,13 +1583,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>195</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1547,13 +1597,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>196</v>
+        <v>163</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1561,13 +1611,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>243</v>
+        <v>165</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1575,13 +1625,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>197</v>
+        <v>166</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1589,13 +1639,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1603,13 +1653,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>199</v>
+        <v>168</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1617,13 +1667,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C27" s="7">
-        <v>1051330011</v>
+        <v>101</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>169</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1631,13 +1681,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>201</v>
+        <v>102</v>
+      </c>
+      <c r="C28" s="5">
+        <v>1051330011</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1645,13 +1695,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>155</v>
+        <v>28</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>202</v>
+        <v>220</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1659,41 +1709,41 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>156</v>
+        <v>30</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>205</v>
+        <v>171</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1701,13 +1751,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>32</v>
+        <v>172</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>206</v>
+        <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1715,27 +1765,27 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>207</v>
+        <v>33</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1743,13 +1793,13 @@
         <v>34</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>209</v>
+        <v>174</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1757,13 +1807,13 @@
         <v>35</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1771,321 +1821,321 @@
         <v>36</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>211</v>
+        <v>176</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>212</v>
+      <c r="B39" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>213</v>
+      <c r="B40" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
+      <c r="B41" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>215</v>
+      <c r="B42" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B43" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>216</v>
+      <c r="B43" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>217</v>
+      <c r="B44" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="6" t="s">
+      <c r="B45" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>219</v>
+      <c r="B46" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>220</v>
+      <c r="B47" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
+      <c r="A48" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B48" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>221</v>
+      <c r="B48" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>222</v>
+      <c r="B49" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>223</v>
+      <c r="B50" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>224</v>
+      <c r="B51" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="D52" s="6" t="s">
-        <v>225</v>
+      <c r="B52" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D52" s="8" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="4" t="s">
+      <c r="A53" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B53" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>226</v>
+      <c r="B53" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C54" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="D54" s="6" t="s">
-        <v>227</v>
+      <c r="B54" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>228</v>
+      <c r="B55" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="6">
-        <v>22</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>164</v>
+      <c r="A56" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>180</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>164</v>
+      <c r="A57" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>180</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>229</v>
+        <v>180</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="4" t="s">
-        <v>57</v>
+      <c r="A60" s="4">
+        <v>22</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>231</v>
+        <v>181</v>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -2093,13 +2143,13 @@
         <v>58</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>232</v>
+        <v>267</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -2107,13 +2157,13 @@
         <v>59</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -2121,13 +2171,13 @@
         <v>60</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -2135,83 +2185,195 @@
         <v>61</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>130</v>
+        <v>262</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>235</v>
+        <v>61</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="6" t="s">
+      <c r="A65" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B65" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="C65" s="7" t="s">
-        <v>169</v>
+      <c r="B65" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>183</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="4" t="s">
+      <c r="A66" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B66" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C66" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>237</v>
+      <c r="B66" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="6" t="s">
+      <c r="A67" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="C67" s="7" t="s">
-        <v>172</v>
+      <c r="B67" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>185</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="4" t="s">
+      <c r="A68" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C68" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="9" t="s">
+      <c r="B68" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="D68" s="8" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B69" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="C69" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="D69" s="9" t="s">
-        <v>240</v>
+      <c r="B69" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D70" s="8" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#18 eSpark and JLCPCB BOM Updated Acc to new Changes
</commit_message>
<xml_diff>
--- a/BOM/JLCPCB-BOM.xlsx
+++ b/BOM/JLCPCB-BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="273">
   <si>
     <t>Comment</t>
   </si>
@@ -99,6 +99,9 @@
     <t>MMZ2012R102ATD25</t>
   </si>
   <si>
+    <t>BLM15PD121SN1D</t>
+  </si>
+  <si>
     <t>10118194-0001LF</t>
   </si>
   <si>
@@ -240,7 +243,7 @@
     <t>CP2102N-A02-GQFN24R</t>
   </si>
   <si>
-    <t>LMV321AIDBVR</t>
+    <t>TLV9301IDCKR</t>
   </si>
   <si>
     <t>X322516MLB4SI</t>
@@ -249,7 +252,7 @@
     <t>Designator</t>
   </si>
   <si>
-    <t>C1</t>
+    <t>C1, C60, C61</t>
   </si>
   <si>
     <t>C2, C7, C9, C10, C12, C13, C19, C20, C21, C22, C29, C30, C31, C32, C33, C34, C35, C37, C40, C41, C44, C45, C46, C47, C48, C49, C51, C54, C56, C57</t>
@@ -267,7 +270,7 @@
     <t>C11, C14, C15, C16, C17, C18, C23, C24, C25, C26, C27, C28</t>
   </si>
   <si>
-    <t>C38, C55</t>
+    <t>C38, C55, C62</t>
   </si>
   <si>
     <t>C39</t>
@@ -324,6 +327,9 @@
     <t>FB2, FB3, FB4, FB5, FB6, FB7, FB8, FB9</t>
   </si>
   <si>
+    <t>FB10</t>
+  </si>
+  <si>
     <t>J1, J2</t>
   </si>
   <si>
@@ -528,6 +534,9 @@
     <t>Ind-0805</t>
   </si>
   <si>
+    <t>IND-0402</t>
+  </si>
+  <si>
     <t>10118194-0001LF_</t>
   </si>
   <si>
@@ -597,7 +606,7 @@
     <t>24-QFN (4x4)</t>
   </si>
   <si>
-    <t>SOT-23-5</t>
+    <t>SC-70-5</t>
   </si>
   <si>
     <t>SMD3225-4P</t>
@@ -675,6 +684,9 @@
     <t>C307765</t>
   </si>
   <si>
+    <t>C76891</t>
+  </si>
+  <si>
     <t>C132563</t>
   </si>
   <si>
@@ -693,6 +705,9 @@
     <t>C492442</t>
   </si>
   <si>
+    <t>C492441</t>
+  </si>
+  <si>
     <t>C597972</t>
   </si>
   <si>
@@ -801,7 +816,7 @@
     <t>C969151</t>
   </si>
   <si>
-    <t>C484730</t>
+    <t>C4366617</t>
   </si>
   <si>
     <t>C13738</t>
@@ -810,13 +825,13 @@
     <t>SB1, SB2, SB8</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>C526997</t>
   </si>
   <si>
     <t>C69679</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>C114765</t>
@@ -1289,7 +1304,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1303,13 +1318,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1317,13 +1332,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="36" x14ac:dyDescent="0.25">
@@ -1331,13 +1346,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1345,13 +1360,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1359,13 +1374,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1373,13 +1388,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1387,13 +1402,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1401,13 +1416,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1415,13 +1430,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1429,13 +1444,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1443,13 +1458,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1457,13 +1472,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1471,13 +1486,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1485,13 +1500,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1499,13 +1514,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1513,13 +1528,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1527,13 +1542,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1541,13 +1556,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1555,13 +1570,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1569,13 +1584,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1583,13 +1598,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1597,13 +1612,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1611,13 +1626,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1625,13 +1640,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1639,13 +1654,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1653,13 +1668,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1667,13 +1682,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1681,13 +1696,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C28" s="5">
-        <v>1051330011</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>219</v>
+        <v>103</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1695,13 +1710,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>220</v>
+        <v>104</v>
+      </c>
+      <c r="C29" s="7">
+        <v>1051330011</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1709,13 +1724,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>221</v>
+        <v>29</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1723,41 +1738,41 @@
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>173</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>38</v>
+        <v>174</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1765,13 +1780,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>224</v>
+        <v>175</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1779,27 +1794,27 @@
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>225</v>
+        <v>34</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>226</v>
+        <v>176</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1807,13 +1822,13 @@
         <v>35</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>227</v>
+        <v>177</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1821,13 +1836,13 @@
         <v>36</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>228</v>
+        <v>178</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1835,13 +1850,13 @@
         <v>37</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>229</v>
+        <v>179</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1849,13 +1864,13 @@
         <v>38</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>265</v>
+        <v>179</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1863,13 +1878,13 @@
         <v>39</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>265</v>
+        <v>180</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1877,13 +1892,13 @@
         <v>40</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>265</v>
+        <v>180</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1891,13 +1906,13 @@
         <v>41</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>230</v>
+        <v>181</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1905,13 +1920,13 @@
         <v>42</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>231</v>
+        <v>182</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1919,41 +1934,41 @@
         <v>43</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>44</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>234</v>
+        <v>183</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1961,13 +1976,13 @@
         <v>46</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>235</v>
+        <v>183</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1975,13 +1990,13 @@
         <v>47</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>236</v>
+        <v>183</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1989,13 +2004,13 @@
         <v>48</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>237</v>
+        <v>183</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -2003,13 +2018,13 @@
         <v>49</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>238</v>
+        <v>183</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -2017,13 +2032,13 @@
         <v>50</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>239</v>
+        <v>183</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -2031,13 +2046,13 @@
         <v>51</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>240</v>
+        <v>183</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -2045,13 +2060,13 @@
         <v>52</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D54" s="8" t="s">
-        <v>241</v>
+        <v>183</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -2059,13 +2074,13 @@
         <v>53</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>242</v>
+        <v>183</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2073,13 +2088,13 @@
         <v>54</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>243</v>
+        <v>183</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -2087,13 +2102,13 @@
         <v>55</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>244</v>
+        <v>183</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -2101,13 +2116,13 @@
         <v>56</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>245</v>
+        <v>183</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -2115,41 +2130,41 @@
         <v>57</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>246</v>
+        <v>183</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="4">
+      <c r="A60" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="6">
         <v>22</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="D60" s="8" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="6" t="s">
-        <v>58</v>
-      </c>
       <c r="B61" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="D61" s="6" t="s">
-        <v>267</v>
+        <v>184</v>
+      </c>
+      <c r="D61" s="8" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -2157,13 +2172,13 @@
         <v>59</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>247</v>
+        <v>184</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -2171,13 +2186,13 @@
         <v>60</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D63" s="6" t="s">
-        <v>248</v>
+        <v>185</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -2185,27 +2200,27 @@
         <v>61</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>262</v>
+        <v>139</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D64" s="9" t="s">
-        <v>265</v>
+        <v>183</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="4" t="s">
+      <c r="A65" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B65" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>249</v>
+      <c r="B65" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -2213,13 +2228,13 @@
         <v>63</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>250</v>
+        <v>186</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -2227,13 +2242,13 @@
         <v>64</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>251</v>
+        <v>187</v>
+      </c>
+      <c r="D67" s="8" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2241,13 +2256,13 @@
         <v>65</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>252</v>
+        <v>188</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2255,13 +2270,13 @@
         <v>66</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="D69" s="6" t="s">
-        <v>253</v>
+        <v>189</v>
+      </c>
+      <c r="D69" s="8" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2269,13 +2284,13 @@
         <v>67</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>254</v>
+        <v>190</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -2283,13 +2298,13 @@
         <v>68</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>255</v>
+        <v>191</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2297,13 +2312,13 @@
         <v>69</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="D72" s="6" t="s">
-        <v>256</v>
+        <v>192</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2311,13 +2326,13 @@
         <v>70</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>257</v>
+        <v>190</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2325,13 +2340,13 @@
         <v>71</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="D74" s="6" t="s">
-        <v>258</v>
+        <v>71</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -2339,13 +2354,13 @@
         <v>72</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>259</v>
+        <v>193</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -2353,13 +2368,13 @@
         <v>73</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="D76" s="6" t="s">
-        <v>260</v>
+        <v>194</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -2367,13 +2382,27 @@
         <v>74</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="D77" s="6" t="s">
-        <v>261</v>
+        <v>195</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#18 2.2uf Capacitor Designator Updated in BOMs
</commit_message>
<xml_diff>
--- a/BOM/JLCPCB-BOM.xlsx
+++ b/BOM/JLCPCB-BOM.xlsx
@@ -285,9 +285,6 @@
     <t>C53</t>
   </si>
   <si>
-    <t>C58, C59</t>
-  </si>
-  <si>
     <t>D1, D2, D3, D17, D18, D23, D24</t>
   </si>
   <si>
@@ -838,6 +835,9 @@
   </si>
   <si>
     <t>C60491</t>
+  </si>
+  <si>
+    <t>Cx3, Cx4</t>
   </si>
 </sst>
 </file>
@@ -1321,10 +1321,10 @@
         <v>76</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1335,10 +1335,10 @@
         <v>77</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="36" x14ac:dyDescent="0.25">
@@ -1349,10 +1349,10 @@
         <v>78</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1363,10 +1363,10 @@
         <v>79</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1377,10 +1377,10 @@
         <v>80</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1391,10 +1391,10 @@
         <v>81</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1405,10 +1405,10 @@
         <v>82</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1419,10 +1419,10 @@
         <v>83</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1433,10 +1433,10 @@
         <v>84</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1447,10 +1447,10 @@
         <v>85</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1461,10 +1461,10 @@
         <v>86</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1475,10 +1475,10 @@
         <v>87</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1486,13 +1486,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>88</v>
+        <v>272</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1500,13 +1500,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1514,13 +1514,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1528,13 +1528,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1542,13 +1542,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1556,13 +1556,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1570,13 +1570,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1584,13 +1584,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1598,13 +1598,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1612,13 +1612,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1626,13 +1626,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1640,13 +1640,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1654,13 +1654,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1668,13 +1668,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1682,13 +1682,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1696,13 +1696,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1710,13 +1710,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C29" s="7">
         <v>1051330011</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1724,13 +1724,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1738,13 +1738,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1752,13 +1752,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1766,13 +1766,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1780,13 +1780,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1794,13 +1794,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1808,13 +1808,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1822,13 +1822,13 @@
         <v>35</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1836,13 +1836,13 @@
         <v>36</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1850,13 +1850,13 @@
         <v>37</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1864,13 +1864,13 @@
         <v>38</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1878,13 +1878,13 @@
         <v>39</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1892,13 +1892,13 @@
         <v>40</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1906,13 +1906,13 @@
         <v>41</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1920,13 +1920,13 @@
         <v>42</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1934,13 +1934,13 @@
         <v>43</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1948,13 +1948,13 @@
         <v>44</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1962,13 +1962,13 @@
         <v>45</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1976,13 +1976,13 @@
         <v>46</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1990,13 +1990,13 @@
         <v>47</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -2004,13 +2004,13 @@
         <v>48</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -2018,13 +2018,13 @@
         <v>49</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -2032,13 +2032,13 @@
         <v>50</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -2046,13 +2046,13 @@
         <v>51</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -2060,13 +2060,13 @@
         <v>52</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -2074,13 +2074,13 @@
         <v>53</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2088,13 +2088,13 @@
         <v>54</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -2102,13 +2102,13 @@
         <v>55</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -2116,13 +2116,13 @@
         <v>56</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -2130,13 +2130,13 @@
         <v>57</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -2144,13 +2144,13 @@
         <v>58</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -2158,13 +2158,13 @@
         <v>22</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -2172,13 +2172,13 @@
         <v>59</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -2186,13 +2186,13 @@
         <v>60</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -2200,13 +2200,13 @@
         <v>61</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -2214,13 +2214,13 @@
         <v>62</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C65" s="7" t="s">
         <v>62</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -2228,13 +2228,13 @@
         <v>63</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -2242,13 +2242,13 @@
         <v>64</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2256,13 +2256,13 @@
         <v>65</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2270,13 +2270,13 @@
         <v>66</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2284,13 +2284,13 @@
         <v>67</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -2298,13 +2298,13 @@
         <v>68</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2312,13 +2312,13 @@
         <v>69</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2326,13 +2326,13 @@
         <v>70</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2340,13 +2340,13 @@
         <v>71</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C74" s="7" t="s">
         <v>71</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -2354,13 +2354,13 @@
         <v>72</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -2368,13 +2368,13 @@
         <v>73</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -2382,13 +2382,13 @@
         <v>74</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -2396,13 +2396,13 @@
         <v>75</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#18 eSpark, CLient and JLCPCB BOM updated
</commit_message>
<xml_diff>
--- a/BOM/JLCPCB-BOM.xlsx
+++ b/BOM/JLCPCB-BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="274">
   <si>
     <t>Comment</t>
   </si>
@@ -255,9 +255,6 @@
     <t>C1, C60, C61</t>
   </si>
   <si>
-    <t>C2, C7, C9, C10, C12, C13, C19, C20, C21, C22, C29, C30, C31, C32, C33, C34, C35, C37, C40, C41, C44, C45, C46, C47, C48, C49, C51, C54, C56, C57</t>
-  </si>
-  <si>
     <t>C3, C5</t>
   </si>
   <si>
@@ -366,12 +363,6 @@
     <t>LED4, LED6, LED8, LED9</t>
   </si>
   <si>
-    <t>LED7</t>
-  </si>
-  <si>
-    <t>LED10</t>
-  </si>
-  <si>
     <t>P1, P2, P3, P4, P5, P6</t>
   </si>
   <si>
@@ -558,9 +549,6 @@
     <t>LED-0603</t>
   </si>
   <si>
-    <t>ZIO-101954</t>
-  </si>
-  <si>
     <t>Test-point</t>
   </si>
   <si>
@@ -819,9 +807,6 @@
     <t>C13738</t>
   </si>
   <si>
-    <t>SB1, SB2, SB8</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -838,6 +823,24 @@
   </si>
   <si>
     <t>Cx3, Cx4</t>
+  </si>
+  <si>
+    <t>C2, C7, C9, C10, C12, C13, C19, C20, C21, C22, C29, C30, C31, C32, C33, C34, C35, C37, C40, C41, C44, C45, C46, C47, C48, C49, C51, C54, Cx1, Cx2</t>
+  </si>
+  <si>
+    <t>OLED7</t>
+  </si>
+  <si>
+    <t>OLED10</t>
+  </si>
+  <si>
+    <t>SB1, SB2 ,SB8</t>
+  </si>
+  <si>
+    <t>C2718488</t>
+  </si>
+  <si>
+    <t>HDRX4</t>
   </si>
 </sst>
 </file>
@@ -988,7 +991,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1015,6 +1018,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1321,52 +1327,52 @@
         <v>76</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="8" t="s">
         <v>77</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="36" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>78</v>
+      <c r="B3" s="10" t="s">
+        <v>268</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>79</v>
+      <c r="B4" s="8" t="s">
+        <v>78</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1374,41 +1380,41 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>81</v>
+      <c r="B6" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>82</v>
+      <c r="B7" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1416,55 +1422,55 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>84</v>
+      <c r="B9" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>85</v>
+      <c r="B10" s="8" t="s">
+        <v>84</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>86</v>
+      <c r="B11" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1472,13 +1478,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1486,195 +1492,195 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>88</v>
+      <c r="B14" s="8" t="s">
+        <v>87</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>89</v>
+      <c r="B15" s="10" t="s">
+        <v>88</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>90</v>
+      <c r="B16" s="8" t="s">
+        <v>89</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>91</v>
+      <c r="B17" s="10" t="s">
+        <v>90</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>92</v>
+      <c r="B18" s="8" t="s">
+        <v>91</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>93</v>
+      <c r="B19" s="10" t="s">
+        <v>92</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>94</v>
+      <c r="B20" s="8" t="s">
+        <v>93</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>95</v>
+      <c r="B21" s="10" t="s">
+        <v>94</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>96</v>
+      <c r="B22" s="8" t="s">
+        <v>95</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>97</v>
+      <c r="B23" s="10" t="s">
+        <v>96</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>98</v>
+      <c r="B24" s="8" t="s">
+        <v>97</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>99</v>
+      <c r="B25" s="10" t="s">
+        <v>98</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>100</v>
+      <c r="B26" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1682,195 +1688,195 @@
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>102</v>
+      <c r="B28" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>103</v>
+      <c r="B29" s="8" t="s">
+        <v>102</v>
       </c>
       <c r="C29" s="7">
         <v>1051330011</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>104</v>
+      <c r="B30" s="10" t="s">
+        <v>103</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>105</v>
+      <c r="B31" s="8" t="s">
+        <v>104</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>106</v>
+      <c r="B32" s="10" t="s">
+        <v>105</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>107</v>
+      <c r="B33" s="8" t="s">
+        <v>106</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>108</v>
+      <c r="B34" s="10" t="s">
+        <v>107</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>109</v>
+      <c r="B35" s="8" t="s">
+        <v>108</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="4" t="s">
-        <v>110</v>
+      <c r="B36" s="10" t="s">
+        <v>109</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>111</v>
+      <c r="B37" s="8" t="s">
+        <v>110</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>112</v>
+      <c r="B38" s="10" t="s">
+        <v>111</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>113</v>
+      <c r="B39" s="8" t="s">
+        <v>112</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>114</v>
+      <c r="B40" s="10" t="s">
+        <v>113</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1878,13 +1884,13 @@
         <v>39</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>115</v>
+        <v>269</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>179</v>
+        <v>273</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1892,517 +1898,517 @@
         <v>40</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>179</v>
+        <v>270</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>273</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>117</v>
+      <c r="B43" s="9" t="s">
+        <v>114</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>118</v>
+      <c r="B44" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="6" t="s">
-        <v>119</v>
+      <c r="B45" s="8" t="s">
+        <v>116</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>120</v>
+      <c r="B46" s="10" t="s">
+        <v>117</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="6" t="s">
-        <v>121</v>
+      <c r="B47" s="8" t="s">
+        <v>118</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>122</v>
+      <c r="B48" s="10" t="s">
+        <v>119</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="6" t="s">
-        <v>123</v>
+      <c r="B49" s="8" t="s">
+        <v>120</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>124</v>
+      <c r="B50" s="10" t="s">
+        <v>121</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B51" s="6" t="s">
-        <v>125</v>
+      <c r="B51" s="8" t="s">
+        <v>122</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="4" t="s">
-        <v>126</v>
+      <c r="B52" s="10" t="s">
+        <v>123</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B53" s="6" t="s">
-        <v>127</v>
+      <c r="B53" s="8" t="s">
+        <v>124</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="4" t="s">
-        <v>128</v>
+      <c r="B54" s="10" t="s">
+        <v>125</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>129</v>
+      <c r="B55" s="8" t="s">
+        <v>126</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B56" s="4" t="s">
-        <v>130</v>
+      <c r="B56" s="10" t="s">
+        <v>127</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B57" s="6" t="s">
-        <v>131</v>
+      <c r="B57" s="8" t="s">
+        <v>128</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>132</v>
+      <c r="B58" s="10" t="s">
+        <v>129</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>133</v>
+      <c r="B59" s="8" t="s">
+        <v>130</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>134</v>
+      <c r="B60" s="10" t="s">
+        <v>131</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="6">
         <v>22</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>135</v>
+      <c r="B61" s="8" t="s">
+        <v>132</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B62" s="4" t="s">
-        <v>136</v>
+      <c r="B62" s="10" t="s">
+        <v>133</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>137</v>
+      <c r="B63" s="4" t="s">
+        <v>134</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B64" s="4" t="s">
-        <v>138</v>
+      <c r="B64" s="6" t="s">
+        <v>135</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B65" s="6" t="s">
-        <v>266</v>
+      <c r="B65" s="9" t="s">
+        <v>271</v>
       </c>
       <c r="C65" s="7" t="s">
         <v>62</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B66" s="6" t="s">
-        <v>139</v>
+      <c r="B66" s="10" t="s">
+        <v>136</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="4" t="s">
-        <v>140</v>
+      <c r="B67" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>141</v>
+      <c r="B68" s="10" t="s">
+        <v>138</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B69" s="4" t="s">
-        <v>142</v>
+      <c r="B69" s="8" t="s">
+        <v>139</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B70" s="6" t="s">
-        <v>143</v>
+      <c r="B70" s="10" t="s">
+        <v>140</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B71" s="4" t="s">
-        <v>144</v>
+      <c r="B71" s="8" t="s">
+        <v>141</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B72" s="6" t="s">
-        <v>145</v>
+      <c r="B72" s="4" t="s">
+        <v>142</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B73" s="4" t="s">
-        <v>146</v>
+      <c r="B73" s="10" t="s">
+        <v>143</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B74" s="6" t="s">
-        <v>147</v>
+      <c r="B74" s="8" t="s">
+        <v>144</v>
       </c>
       <c r="C74" s="7" t="s">
         <v>71</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B75" s="4" t="s">
-        <v>148</v>
+      <c r="B75" s="10" t="s">
+        <v>145</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B76" s="6" t="s">
-        <v>149</v>
+      <c r="B76" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B77" s="4" t="s">
-        <v>150</v>
+      <c r="B77" s="6" t="s">
+        <v>147</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B78" s="6" t="s">
-        <v>151</v>
+      <c r="B78" s="10" t="s">
+        <v>148</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>